<commit_message>
Refactor DSA rates and job grades in tests and views
- Updated job grades from 'NGCDF X' format to numeric format in various tests and views for consistency.
- Introduced DocumentFont support for PDF generation in reports, ensuring proper font usage.
- Added tests for DocumentFont functionality and DSA standard rates calculations.
- Adjusted DSA rate creation in tests to reflect new job grade format.
- Cleaned up unused County model references in tests.
- Ensured proper handling of DSA rates in import and export functionalities.
</commit_message>
<xml_diff>
--- a/docs/hr-import/HR-Staff-Import-Template.xlsx
+++ b/docs/hr-import/HR-Staff-Import-Template.xlsx
@@ -6529,7 +6529,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Employment Type" error="Choose a Employment Type from the list (see the Lists sheet)." type="list">
       <formula1>=Lists!$A$2:$A$4</formula1>
     </dataValidation>
@@ -6541,6 +6541,9 @@
     </dataValidation>
     <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Active" error="Choose a Active from the list (see the Lists sheet)." type="list">
       <formula1>=Lists!$D$2:$D$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Job Grade" error="Choose the scale from the HR register (1 to 10), or INTERN for casuals and attachees." type="list">
+      <formula1>=Lists!$E$2:$E$12</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6659,7 +6662,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Job Grade: e.g. NGCDF 6. It sets the officer's DSA rate, so it must match a grade in Settings &gt; DSA rates.</t>
+          <t>Job Grade: the officer's scale from the HR staff register (Job Scale), 1 to 10. It sets the DSA rate: one standard rate per scale, wherever the activity is. INTERN is for casuals and attachees only, and a casual or attachee left blank gets INTERN. A column headed "Job Scale" is read too. A blank cell never erases a scale already in the system.</t>
         </is>
       </c>
     </row>
@@ -6726,13 +6729,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6756,6 +6760,11 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Job Grade</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6778,6 +6787,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6800,6 +6812,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6817,6 +6832,9 @@
           <t>Coast Region</t>
         </is>
       </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
@@ -6829,6 +6847,9 @@
           <t>Lower Eastern Region</t>
         </is>
       </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
@@ -6841,6 +6862,9 @@
           <t>Nairobi Region</t>
         </is>
       </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
@@ -6853,6 +6877,9 @@
           <t>North Eastern Region</t>
         </is>
       </c>
+      <c r="E7" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
@@ -6865,6 +6892,9 @@
           <t>North Rift Region</t>
         </is>
       </c>
+      <c r="E8" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
@@ -6877,6 +6907,9 @@
           <t>Nyanza Region</t>
         </is>
       </c>
+      <c r="E9" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
@@ -6889,6 +6922,9 @@
           <t>South Rift Region</t>
         </is>
       </c>
+      <c r="E10" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
@@ -6901,6 +6937,9 @@
           <t>Upper Eastern Region</t>
         </is>
       </c>
+      <c r="E11" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
@@ -6911,6 +6950,11 @@
       <c r="C12" t="inlineStr">
         <is>
           <t>Western Region</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>INTERN</t>
         </is>
       </c>
     </row>

</xml_diff>